<commit_message>
working on making PC scenarios
</commit_message>
<xml_diff>
--- a/DATA/Starting_point.xlsx
+++ b/DATA/Starting_point.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30A8FEE2-BE8F-4FE6-A73D-C8D61511F8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{30A8FEE2-BE8F-4FE6-A73D-C8D61511F8D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8894626D-86F3-4941-8085-00703CF562E5}"/>
   <bookViews>
-    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="F_start" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="39">
   <si>
     <t>Measles</t>
   </si>
@@ -1137,7 +1137,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFBA2FAA-95C5-423D-A8C0-3A912D67D407}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1178,6 +1178,86 @@
       </c>
       <c r="B5">
         <v>5145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1190,8 +1270,7 @@
   <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>